<commit_message>
cafe-app: fictional realistic names in the test-data kit (one identity per person across files)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3ov37P2fF1cuhtF4wyed3
</commit_message>
<xml_diff>
--- a/cafe-app/test-data/01-submissions.xlsx
+++ b/cafe-app/test-data/01-submissions.xlsx
@@ -52,7 +52,7 @@
     <t>Vendor contract summariser</t>
   </si>
   <si>
-    <t>Person 1 (CS)</t>
+    <t>Avery Chen (CS)</t>
   </si>
   <si>
     <t>Legal Ops</t>
@@ -85,7 +85,7 @@
     <t>Desk booking assistant</t>
   </si>
   <si>
-    <t>Person 2 (CS)</t>
+    <t>Priya Nair (CS)</t>
   </si>
   <si>
     <t>Workplace</t>
@@ -97,7 +97,7 @@
     <t>Team</t>
   </si>
   <si>
-    <t>Person 2 (Lead); Person 3 (Sponsor); Person 9</t>
+    <t>Priya Nair (Lead); Tomasz Wiśniewski (Sponsor); Rhys Llewellyn</t>
   </si>
   <si>
     <t>Staff cannot easily see which desks are free and often book ones that are already taken.</t>
@@ -118,7 +118,7 @@
     <t>Onboarding checklist helper</t>
   </si>
   <si>
-    <t>Person 5 (CS)</t>
+    <t>Mateo Álvarez (CS)</t>
   </si>
   <si>
     <t>BSI</t>
@@ -142,13 +142,13 @@
     <t>Expense anomaly finder</t>
   </si>
   <si>
-    <t>Person 6 (CS)</t>
+    <t>Ingrid Solberg (CS)</t>
   </si>
   <si>
     <t>GSS</t>
   </si>
   <si>
-    <t>Person 6 (Lead); Person 4 (Sponsor); Person 8</t>
+    <t>Ingrid Solberg (Lead); Noor El-Sayed (Sponsor); Hana Kobayashi</t>
   </si>
   <si>
     <t>Unusual expense claims are only spotted when a reviewer happens to notice them.</t>
@@ -166,7 +166,7 @@
     <t>Meeting notes to actions</t>
   </si>
   <si>
-    <t>Person 10 (CS)</t>
+    <t>Zainab Okafor (CS)</t>
   </si>
   <si>
     <t>Actions agreed in meetings are lost because nobody writes them up the same day.</t>
@@ -184,7 +184,7 @@
     <t>Travel policy assistant</t>
   </si>
   <si>
-    <t>Person 11 (CS)</t>
+    <t>Lucía Fernández (CS)</t>
   </si>
   <si>
     <t>Travellers keep asking the same questions about what the travel policy allows.</t>
@@ -199,7 +199,7 @@
     <t>;#Agent Design Guidance;#</t>
   </si>
   <si>
-    <t>Person 12 (CS)</t>
+    <t>Dmitri Volkov (CS)</t>
   </si>
   <si>
     <t>Facilities requests arrive by phone, email and chat and are sorted by hand.</t>
@@ -214,10 +214,10 @@
     <t>Procurement FAQ bot</t>
   </si>
   <si>
-    <t>Person 7 (CS)</t>
-  </si>
-  <si>
-    <t>Person 7 (Lead); Person 1 (Sponsor); Person 10</t>
+    <t>Kwame Mensah (CS)</t>
+  </si>
+  <si>
+    <t>Kwame Mensah (Lead); Avery Chen (Sponsor); Zainab Okafor</t>
   </si>
   <si>
     <t>Business teams ask procurement the same questions about thresholds and approved suppliers.</t>

</xml_diff>